<commit_message>
employee attendace report new api and user import new field added
</commit_message>
<xml_diff>
--- a/Presentation/AVPolyPack.API/FormatFiles/Template_User.xlsx
+++ b/Presentation/AVPolyPack.API/FormatFiles/Template_User.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="99">
   <si>
     <t>UserCode</t>
   </si>
@@ -110,9 +110,6 @@
     <t>5566998877</t>
   </si>
   <si>
-    <t>email1@gmail.com</t>
-  </si>
-  <si>
     <t>123</t>
   </si>
   <si>
@@ -173,9 +170,6 @@
     <t>2336655444</t>
   </si>
   <si>
-    <t>email2@gmail.com</t>
-  </si>
-  <si>
     <t>12334</t>
   </si>
   <si>
@@ -219,13 +213,124 @@
   </si>
   <si>
     <t>vmfkvnfbjsk=</t>
+  </si>
+  <si>
+    <t>EmployeeType</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>MaritalStatus</t>
+  </si>
+  <si>
+    <t>WorkingHour</t>
+  </si>
+  <si>
+    <t>Rate</t>
+  </si>
+  <si>
+    <t>RateValue</t>
+  </si>
+  <si>
+    <t>EmergencyName</t>
+  </si>
+  <si>
+    <t>EmergencyRelation</t>
+  </si>
+  <si>
+    <t>BankName</t>
+  </si>
+  <si>
+    <t>BankAccountNo</t>
+  </si>
+  <si>
+    <t>BankIFSCCode</t>
+  </si>
+  <si>
+    <t>OtherProof</t>
+  </si>
+  <si>
+    <t>IsSupervisor</t>
+  </si>
+  <si>
+    <t>Contract</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>xyz</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Son</t>
+  </si>
+  <si>
+    <t>Father</t>
+  </si>
+  <si>
+    <t>Married</t>
+  </si>
+  <si>
+    <t>Unmarried</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Daily Rate</t>
+  </si>
+  <si>
+    <t>Monthly Rate</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>130</t>
+  </si>
+  <si>
+    <t>SBI</t>
+  </si>
+  <si>
+    <t>Central</t>
+  </si>
+  <si>
+    <t>SBI101</t>
+  </si>
+  <si>
+    <t>C101</t>
+  </si>
+  <si>
+    <t>TestProof</t>
+  </si>
+  <si>
+    <t>abc@gmail.com</t>
+  </si>
+  <si>
+    <t>test@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -239,12 +344,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -294,7 +393,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -314,23 +413,23 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -604,512 +703,703 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X49"/>
+  <dimension ref="A1:AL49"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="13.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="2" customWidth="1"/>
-    <col min="4" max="4" width="16" style="3" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="20.85546875" style="3" customWidth="1"/>
-    <col min="7" max="7" width="18.28515625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="16.5703125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" style="3" customWidth="1"/>
-    <col min="11" max="11" width="8" style="2" customWidth="1"/>
-    <col min="12" max="12" width="14.42578125" style="2" customWidth="1"/>
-    <col min="13" max="14" width="8" style="2" customWidth="1"/>
-    <col min="15" max="15" width="11.7109375" style="2" customWidth="1"/>
-    <col min="16" max="16" width="13.5703125" style="2" customWidth="1"/>
-    <col min="17" max="17" width="25.28515625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="11.7109375" style="2" customWidth="1"/>
-    <col min="19" max="20" width="14.5703125" style="2" customWidth="1"/>
-    <col min="21" max="21" width="15.28515625" style="2" customWidth="1"/>
-    <col min="22" max="22" width="12.7109375" customWidth="1"/>
-    <col min="23" max="23" width="10.7109375" customWidth="1"/>
-    <col min="24" max="24" width="8" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="20.85546875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="18.28515625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="16.5703125" style="3" customWidth="1"/>
+    <col min="11" max="12" width="10.7109375" style="3" customWidth="1"/>
+    <col min="13" max="13" width="10.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.42578125" style="2" customWidth="1"/>
+    <col min="15" max="15" width="14.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8" style="2" customWidth="1"/>
+    <col min="17" max="17" width="11.7109375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="13.5703125" style="2" customWidth="1"/>
+    <col min="19" max="19" width="16.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="25.28515625" style="2" customWidth="1"/>
+    <col min="22" max="23" width="11.7109375" style="2" customWidth="1"/>
+    <col min="24" max="24" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="27" width="12.85546875" style="2" customWidth="1"/>
+    <col min="28" max="28" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.42578125" style="12" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="14.5703125" style="2" customWidth="1"/>
+    <col min="33" max="33" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.7109375" customWidth="1"/>
+    <col min="35" max="35" width="15.28515625" style="2" customWidth="1"/>
+    <col min="36" max="36" width="12.7109375" customWidth="1"/>
+    <col min="37" max="37" width="10.7109375" customWidth="1"/>
+    <col min="38" max="38" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:38">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="S1" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="T1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="U1" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="V1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="W1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="X1" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y1" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="Z1" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="AA1" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="AB1" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC1" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD1" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="AE1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="AF1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="AG1" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="AH1" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="AI1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="12" t="s">
+      <c r="AJ1" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="12" t="s">
+      <c r="AK1" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="13" t="s">
+      <c r="AL1" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:38">
       <c r="A2" t="s">
         <v>24</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="G2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="H2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="J2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="K2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="L2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="Q2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="S2" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="T2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="U2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="V2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="W2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="AC2" s="12">
+        <v>1122222</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="AF2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="AG2" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="AH2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="AJ2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:38">
+      <c r="A3" t="s">
         <v>44</v>
       </c>
-      <c r="V2" t="b">
+      <c r="B3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Z3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AC3" s="12">
+        <v>2536417</v>
+      </c>
+      <c r="AD3" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AE3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG3" s="3"/>
+      <c r="AH3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AJ3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="b">
         <v>1</v>
       </c>
-      <c r="W2" t="b">
+      <c r="AL3" t="b">
         <v>0</v>
       </c>
-      <c r="X2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24">
-      <c r="A3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="V3" t="b">
-        <v>0</v>
-      </c>
-      <c r="W3" t="b">
-        <v>1</v>
-      </c>
-      <c r="X3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24">
-      <c r="D4" s="9"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="2"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
+    </row>
+    <row r="4" spans="1:38">
+      <c r="I4" s="1"/>
+      <c r="J4" s="2"/>
       <c r="M4" s="3"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="1"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-    </row>
-    <row r="5" spans="1:24">
-      <c r="D5" s="9"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="2"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="1"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="1"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-    </row>
-    <row r="6" spans="1:24">
-      <c r="H6" s="1"/>
-      <c r="I6" s="2"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="1"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="1"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-    </row>
-    <row r="7" spans="1:24">
-      <c r="H7" s="1"/>
-      <c r="I7" s="2"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="1"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="1"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-    </row>
-    <row r="8" spans="1:24">
-      <c r="H8" s="1"/>
-      <c r="I8" s="2"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="1"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="1"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-      <c r="U8" s="3"/>
-    </row>
-    <row r="9" spans="1:24">
-      <c r="H9" s="1"/>
-      <c r="I9" s="2"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="1"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="1"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="3"/>
-    </row>
-    <row r="10" spans="1:24">
-      <c r="H10" s="1"/>
-      <c r="I10" s="2"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="1"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="1"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="3"/>
-    </row>
-    <row r="11" spans="1:24">
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-    </row>
-    <row r="12" spans="1:24">
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-    </row>
-    <row r="13" spans="1:24">
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-    </row>
-    <row r="14" spans="1:24">
-      <c r="O14" s="11"/>
-      <c r="P14" s="11"/>
-    </row>
-    <row r="15" spans="1:24">
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-    </row>
-    <row r="16" spans="1:24">
-      <c r="O16" s="11"/>
-      <c r="P16" s="11"/>
-    </row>
-    <row r="17" spans="15:16">
-      <c r="O17" s="11"/>
-      <c r="P17" s="11"/>
-    </row>
-    <row r="18" spans="15:16">
-      <c r="O18" s="11"/>
-      <c r="P18" s="11"/>
-    </row>
-    <row r="19" spans="15:16">
-      <c r="O19" s="11"/>
-      <c r="P19" s="11"/>
-    </row>
-    <row r="20" spans="15:16">
-      <c r="O20" s="11"/>
-      <c r="P20" s="11"/>
-    </row>
-    <row r="21" spans="15:16">
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-    </row>
-    <row r="22" spans="15:16">
-      <c r="O22" s="11"/>
-      <c r="P22" s="11"/>
-    </row>
-    <row r="23" spans="15:16">
-      <c r="O23" s="11"/>
-      <c r="P23" s="11"/>
-    </row>
-    <row r="24" spans="15:16">
-      <c r="O24" s="11"/>
-      <c r="P24" s="11"/>
-    </row>
-    <row r="25" spans="15:16">
-      <c r="O25" s="11"/>
-      <c r="P25" s="11"/>
-    </row>
-    <row r="26" spans="15:16">
-      <c r="O26" s="11"/>
-      <c r="P26" s="11"/>
-    </row>
-    <row r="27" spans="15:16">
-      <c r="O27" s="11"/>
-      <c r="P27" s="11"/>
-    </row>
-    <row r="28" spans="15:16">
-      <c r="O28" s="11"/>
-      <c r="P28" s="11"/>
-    </row>
-    <row r="29" spans="15:16">
-      <c r="O29" s="11"/>
-      <c r="P29" s="11"/>
-    </row>
-    <row r="30" spans="15:16">
-      <c r="O30" s="11"/>
-      <c r="P30" s="11"/>
-    </row>
-    <row r="31" spans="15:16">
-      <c r="O31" s="11"/>
-      <c r="P31" s="11"/>
-    </row>
-    <row r="32" spans="15:16">
-      <c r="O32" s="11"/>
-      <c r="P32" s="11"/>
-    </row>
-    <row r="33" spans="15:16">
-      <c r="O33" s="11"/>
-      <c r="P33" s="11"/>
-    </row>
-    <row r="34" spans="15:16">
-      <c r="O34" s="11"/>
-      <c r="P34" s="11"/>
-    </row>
-    <row r="35" spans="15:16">
-      <c r="O35" s="11"/>
-      <c r="P35" s="11"/>
-    </row>
-    <row r="36" spans="15:16">
-      <c r="O36" s="11"/>
-      <c r="P36" s="11"/>
-    </row>
-    <row r="37" spans="15:16">
-      <c r="O37" s="11"/>
-      <c r="P37" s="11"/>
-    </row>
-    <row r="38" spans="15:16">
-      <c r="O38" s="11"/>
-      <c r="P38" s="11"/>
-    </row>
-    <row r="39" spans="15:16">
-      <c r="O39" s="11"/>
-      <c r="P39" s="11"/>
-    </row>
-    <row r="40" spans="15:16">
-      <c r="O40" s="11"/>
-      <c r="P40" s="11"/>
-    </row>
-    <row r="41" spans="15:16">
-      <c r="O41" s="11"/>
-      <c r="P41" s="11"/>
-    </row>
-    <row r="42" spans="15:16">
-      <c r="O42" s="11"/>
-      <c r="P42" s="11"/>
-    </row>
-    <row r="43" spans="15:16">
-      <c r="O43" s="11"/>
-      <c r="P43" s="11"/>
-    </row>
-    <row r="44" spans="15:16">
-      <c r="O44" s="11"/>
-      <c r="P44" s="11"/>
-    </row>
-    <row r="45" spans="15:16">
-      <c r="O45" s="11"/>
-      <c r="P45" s="11"/>
-    </row>
-    <row r="46" spans="15:16">
-      <c r="O46" s="11"/>
-      <c r="P46" s="11"/>
-    </row>
-    <row r="47" spans="15:16">
-      <c r="O47" s="11"/>
-      <c r="P47" s="11"/>
-    </row>
-    <row r="48" spans="15:16">
-      <c r="O48" s="11"/>
-      <c r="P48" s="11"/>
-    </row>
-    <row r="49" spans="15:16">
-      <c r="O49" s="11"/>
-      <c r="P49" s="11"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="Q4" s="8"/>
+      <c r="R4" s="8"/>
+      <c r="S4" s="8"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="3"/>
+      <c r="AG4" s="3"/>
+      <c r="AI4" s="3"/>
+    </row>
+    <row r="5" spans="1:38">
+      <c r="I5" s="1"/>
+      <c r="J5" s="2"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="1"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="8"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="AE5" s="3"/>
+      <c r="AF5" s="3"/>
+      <c r="AG5" s="3"/>
+      <c r="AI5" s="3"/>
+    </row>
+    <row r="6" spans="1:38">
+      <c r="I6" s="1"/>
+      <c r="J6" s="2"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="1"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="8"/>
+      <c r="S6" s="8"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="AE6" s="3"/>
+      <c r="AF6" s="3"/>
+      <c r="AG6" s="3"/>
+      <c r="AI6" s="3"/>
+    </row>
+    <row r="7" spans="1:38">
+      <c r="I7" s="1"/>
+      <c r="J7" s="2"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="1"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="8"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="AE7" s="3"/>
+      <c r="AF7" s="3"/>
+      <c r="AG7" s="3"/>
+      <c r="AI7" s="3"/>
+    </row>
+    <row r="8" spans="1:38">
+      <c r="I8" s="1"/>
+      <c r="J8" s="2"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="1"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="AE8" s="3"/>
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="3"/>
+      <c r="AI8" s="3"/>
+    </row>
+    <row r="9" spans="1:38">
+      <c r="I9" s="1"/>
+      <c r="J9" s="2"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="1"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="1"/>
+      <c r="U9" s="1"/>
+      <c r="AE9" s="3"/>
+      <c r="AF9" s="3"/>
+      <c r="AI9" s="3"/>
+    </row>
+    <row r="10" spans="1:38">
+      <c r="I10" s="1"/>
+      <c r="J10" s="2"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="1"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="1"/>
+      <c r="U10" s="1"/>
+      <c r="AE10" s="3"/>
+      <c r="AF10" s="3"/>
+      <c r="AI10" s="3"/>
+    </row>
+    <row r="11" spans="1:38">
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9"/>
+      <c r="S11" s="9"/>
+    </row>
+    <row r="12" spans="1:38">
+      <c r="Q12" s="9"/>
+      <c r="R12" s="9"/>
+      <c r="S12" s="9"/>
+    </row>
+    <row r="13" spans="1:38">
+      <c r="Q13" s="9"/>
+      <c r="R13" s="9"/>
+      <c r="S13" s="9"/>
+    </row>
+    <row r="14" spans="1:38">
+      <c r="Q14" s="9"/>
+      <c r="R14" s="9"/>
+      <c r="S14" s="9"/>
+    </row>
+    <row r="15" spans="1:38">
+      <c r="Q15" s="9"/>
+      <c r="R15" s="9"/>
+      <c r="S15" s="9"/>
+    </row>
+    <row r="16" spans="1:38">
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
+      <c r="S16" s="9"/>
+    </row>
+    <row r="17" spans="17:19">
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9"/>
+      <c r="S17" s="9"/>
+    </row>
+    <row r="18" spans="17:19">
+      <c r="Q18" s="9"/>
+      <c r="R18" s="9"/>
+      <c r="S18" s="9"/>
+    </row>
+    <row r="19" spans="17:19">
+      <c r="Q19" s="9"/>
+      <c r="R19" s="9"/>
+      <c r="S19" s="9"/>
+    </row>
+    <row r="20" spans="17:19">
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9"/>
+      <c r="S20" s="9"/>
+    </row>
+    <row r="21" spans="17:19">
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
+      <c r="S21" s="9"/>
+    </row>
+    <row r="22" spans="17:19">
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9"/>
+      <c r="S22" s="9"/>
+    </row>
+    <row r="23" spans="17:19">
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9"/>
+      <c r="S23" s="9"/>
+    </row>
+    <row r="24" spans="17:19">
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9"/>
+      <c r="S24" s="9"/>
+    </row>
+    <row r="25" spans="17:19">
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9"/>
+      <c r="S25" s="9"/>
+    </row>
+    <row r="26" spans="17:19">
+      <c r="Q26" s="9"/>
+      <c r="R26" s="9"/>
+      <c r="S26" s="9"/>
+    </row>
+    <row r="27" spans="17:19">
+      <c r="Q27" s="9"/>
+      <c r="R27" s="9"/>
+      <c r="S27" s="9"/>
+    </row>
+    <row r="28" spans="17:19">
+      <c r="Q28" s="9"/>
+      <c r="R28" s="9"/>
+      <c r="S28" s="9"/>
+    </row>
+    <row r="29" spans="17:19">
+      <c r="Q29" s="9"/>
+      <c r="R29" s="9"/>
+      <c r="S29" s="9"/>
+    </row>
+    <row r="30" spans="17:19">
+      <c r="Q30" s="9"/>
+      <c r="R30" s="9"/>
+      <c r="S30" s="9"/>
+    </row>
+    <row r="31" spans="17:19">
+      <c r="Q31" s="9"/>
+      <c r="R31" s="9"/>
+      <c r="S31" s="9"/>
+    </row>
+    <row r="32" spans="17:19">
+      <c r="Q32" s="9"/>
+      <c r="R32" s="9"/>
+      <c r="S32" s="9"/>
+    </row>
+    <row r="33" spans="17:19">
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+    </row>
+    <row r="34" spans="17:19">
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+    </row>
+    <row r="35" spans="17:19">
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+    </row>
+    <row r="36" spans="17:19">
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+    </row>
+    <row r="37" spans="17:19">
+      <c r="Q37" s="9"/>
+      <c r="R37" s="9"/>
+      <c r="S37" s="9"/>
+    </row>
+    <row r="38" spans="17:19">
+      <c r="Q38" s="9"/>
+      <c r="R38" s="9"/>
+      <c r="S38" s="9"/>
+    </row>
+    <row r="39" spans="17:19">
+      <c r="Q39" s="9"/>
+      <c r="R39" s="9"/>
+      <c r="S39" s="9"/>
+    </row>
+    <row r="40" spans="17:19">
+      <c r="Q40" s="9"/>
+      <c r="R40" s="9"/>
+      <c r="S40" s="9"/>
+    </row>
+    <row r="41" spans="17:19">
+      <c r="Q41" s="9"/>
+      <c r="R41" s="9"/>
+      <c r="S41" s="9"/>
+    </row>
+    <row r="42" spans="17:19">
+      <c r="Q42" s="9"/>
+      <c r="R42" s="9"/>
+      <c r="S42" s="9"/>
+    </row>
+    <row r="43" spans="17:19">
+      <c r="Q43" s="9"/>
+      <c r="R43" s="9"/>
+      <c r="S43" s="9"/>
+    </row>
+    <row r="44" spans="17:19">
+      <c r="Q44" s="9"/>
+      <c r="R44" s="9"/>
+      <c r="S44" s="9"/>
+    </row>
+    <row r="45" spans="17:19">
+      <c r="Q45" s="9"/>
+      <c r="R45" s="9"/>
+      <c r="S45" s="9"/>
+    </row>
+    <row r="46" spans="17:19">
+      <c r="Q46" s="9"/>
+      <c r="R46" s="9"/>
+      <c r="S46" s="9"/>
+    </row>
+    <row r="47" spans="17:19">
+      <c r="Q47" s="9"/>
+      <c r="R47" s="9"/>
+      <c r="S47" s="9"/>
+    </row>
+    <row r="48" spans="17:19">
+      <c r="Q48" s="9"/>
+      <c r="R48" s="9"/>
+      <c r="S48" s="9"/>
+    </row>
+    <row r="49" spans="17:19">
+      <c r="Q49" s="9"/>
+      <c r="R49" s="9"/>
+      <c r="S49" s="9"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2 W2 V3 W3 X3 V4:V9 V10:V20 V21:V1048576 W4:W9 W10:W20 W21:W1048576 X1:X2 X4:X10 X11:X1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AK1048576 AL1:AL1048576 AH2:AH1048576">
       <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" tooltip="mailto:email1@gmail.com"/>
-    <hyperlink ref="D3" r:id="rId2" tooltip="mailto:email2@gmail.com"/>
+    <hyperlink ref="E2" r:id="rId1"/>
+    <hyperlink ref="E3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
dashboard new api and issue fixed
</commit_message>
<xml_diff>
--- a/Presentation/AVPolyPack.API/FormatFiles/Template_User.xlsx
+++ b/Presentation/AVPolyPack.API/FormatFiles/Template_User.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="93">
   <si>
     <t>UserCode</t>
   </si>
@@ -38,9 +38,6 @@
     <t>MobileNumber</t>
   </si>
   <si>
-    <t>EmailId</t>
-  </si>
-  <si>
     <t>Password</t>
   </si>
   <si>
@@ -89,9 +86,6 @@
     <t>PanNumber</t>
   </si>
   <si>
-    <t>MobileUniqueId</t>
-  </si>
-  <si>
     <t>IsMobileUser</t>
   </si>
   <si>
@@ -155,9 +149,6 @@
     <t>ARMPJ3654N</t>
   </si>
   <si>
-    <t>dfdfsfsnfksdf=</t>
-  </si>
-  <si>
     <t>EMP002</t>
   </si>
   <si>
@@ -209,9 +200,6 @@
     <t>ARMPJ8944W</t>
   </si>
   <si>
-    <t>vmfkvnfbjsk=</t>
-  </si>
-  <si>
     <t>EmployeeType</t>
   </si>
   <si>
@@ -315,12 +303,6 @@
   </si>
   <si>
     <t>TestProof</t>
-  </si>
-  <si>
-    <t>abc@gmail.com</t>
-  </si>
-  <si>
-    <t>test@gmail.com</t>
   </si>
   <si>
     <t>DAYANAND</t>
@@ -330,7 +312,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -360,13 +342,6 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -391,13 +366,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -427,12 +399,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -703,44 +671,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AL49"/>
+  <dimension ref="A1:AJ49"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="13.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="20.85546875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="18.28515625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="16.5703125" style="3" customWidth="1"/>
-    <col min="11" max="12" width="10.7109375" style="3" customWidth="1"/>
-    <col min="13" max="13" width="10.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.42578125" style="2" customWidth="1"/>
-    <col min="15" max="15" width="14.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8" style="2" customWidth="1"/>
-    <col min="17" max="17" width="11.7109375" style="2" customWidth="1"/>
-    <col min="18" max="18" width="13.5703125" style="2" customWidth="1"/>
-    <col min="19" max="19" width="16.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="25.28515625" style="2" customWidth="1"/>
-    <col min="22" max="23" width="11.7109375" style="2" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="27" width="12.85546875" style="2" customWidth="1"/>
-    <col min="28" max="28" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="18.42578125" style="12" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="14.5703125" style="2" customWidth="1"/>
-    <col min="33" max="33" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12.7109375" customWidth="1"/>
-    <col min="35" max="35" width="15.28515625" style="2" customWidth="1"/>
-    <col min="36" max="36" width="12.7109375" customWidth="1"/>
-    <col min="37" max="37" width="10.7109375" customWidth="1"/>
-    <col min="38" max="38" width="8" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="20.85546875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="18.28515625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" style="3" customWidth="1"/>
+    <col min="10" max="11" width="10.7109375" style="3" customWidth="1"/>
+    <col min="12" max="12" width="10.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" style="2" customWidth="1"/>
+    <col min="14" max="14" width="14.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8" style="2" customWidth="1"/>
+    <col min="16" max="16" width="11.7109375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="13.5703125" style="2" customWidth="1"/>
+    <col min="18" max="18" width="16.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="25.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.28515625" style="2" customWidth="1"/>
+    <col min="21" max="22" width="11.7109375" style="2" customWidth="1"/>
+    <col min="23" max="23" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="26" width="12.85546875" style="2" customWidth="1"/>
+    <col min="27" max="27" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.42578125" style="12" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="14.5703125" style="2" customWidth="1"/>
+    <col min="32" max="32" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="12.7109375" customWidth="1"/>
+    <col min="35" max="35" width="10.7109375" customWidth="1"/>
+    <col min="36" max="36" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38">
+    <row r="1" spans="1:36">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -748,12 +713,12 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="6" t="s">
@@ -772,10 +737,10 @@
         <v>8</v>
       </c>
       <c r="K1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>9</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>10</v>
@@ -793,614 +758,585 @@
         <v>14</v>
       </c>
       <c r="R1" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="S1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="T1" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="V1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="W1" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="X1" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="Z1" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA1" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AB1" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="AC1" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="T1" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="U1" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="V1" s="6" t="s">
+      <c r="AD1" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="W1" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="X1" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y1" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z1" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="AA1" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="AB1" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="AC1" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="AD1" s="6" t="s">
-        <v>74</v>
       </c>
       <c r="AE1" s="6" t="s">
         <v>18</v>
       </c>
       <c r="AF1" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="AG1" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="AH1" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="AG1" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH1" s="10" t="s">
+      <c r="AI1" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="AJ1" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="AI1" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="AJ1" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="AK1" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="AL1" s="11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:38">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q2" s="3" t="s">
+      <c r="S2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="T2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="U2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="S2" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="T2" s="2" t="s">
+      <c r="V2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB2" s="12">
+        <v>1122222</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AD2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U2" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="V2" s="2" t="s">
+      <c r="AE2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="W2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AB2" s="2" t="s">
+      <c r="AF2" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="AC2" s="12">
-        <v>1122222</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="AE2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="AF2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG2" s="3" t="s">
-        <v>95</v>
+      <c r="AG2" t="b">
+        <v>1</v>
       </c>
       <c r="AH2" t="b">
         <v>1</v>
       </c>
-      <c r="AI2" s="2" t="s">
-        <v>42</v>
+      <c r="AI2" t="b">
+        <v>0</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
       </c>
-      <c r="AK2" t="b">
+    </row>
+    <row r="3" spans="1:36">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Z3" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AB3" s="12">
+        <v>2536417</v>
+      </c>
+      <c r="AC3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AD3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AE3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF3" s="3"/>
+      <c r="AG3" t="b">
         <v>0</v>
       </c>
-      <c r="AL2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:38">
-      <c r="A3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="S3" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="X3" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="Z3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA3" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="AB3" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="AC3" s="12">
-        <v>2536417</v>
-      </c>
-      <c r="AD3" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AE3" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AF3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AG3" s="3"/>
       <c r="AH3" t="b">
         <v>0</v>
       </c>
-      <c r="AI3" s="2" t="s">
-        <v>60</v>
+      <c r="AI3" t="b">
+        <v>1</v>
       </c>
       <c r="AJ3" t="b">
         <v>0</v>
       </c>
-      <c r="AK3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:38">
-      <c r="I4" s="1"/>
-      <c r="J4" s="2"/>
+    </row>
+    <row r="4" spans="1:36">
+      <c r="H4" s="1"/>
+      <c r="I4" s="2"/>
+      <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
+      <c r="P4" s="8"/>
       <c r="Q4" s="8"/>
       <c r="R4" s="8"/>
-      <c r="S4" s="8"/>
+      <c r="S4" s="1"/>
       <c r="T4" s="1"/>
-      <c r="U4" s="1"/>
+      <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
       <c r="AF4" s="3"/>
-      <c r="AG4" s="3"/>
-      <c r="AI4" s="3"/>
-    </row>
-    <row r="5" spans="1:38">
-      <c r="I5" s="1"/>
-      <c r="J5" s="2"/>
+    </row>
+    <row r="5" spans="1:36">
+      <c r="H5" s="1"/>
+      <c r="I5" s="2"/>
+      <c r="L5" s="3"/>
       <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="P5" s="8"/>
       <c r="Q5" s="8"/>
       <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
+      <c r="S5" s="1"/>
       <c r="T5" s="1"/>
-      <c r="U5" s="1"/>
+      <c r="AD5" s="3"/>
       <c r="AE5" s="3"/>
       <c r="AF5" s="3"/>
-      <c r="AG5" s="3"/>
-      <c r="AI5" s="3"/>
-    </row>
-    <row r="6" spans="1:38">
-      <c r="I6" s="1"/>
-      <c r="J6" s="2"/>
+    </row>
+    <row r="6" spans="1:36">
+      <c r="H6" s="1"/>
+      <c r="I6" s="2"/>
+      <c r="L6" s="3"/>
       <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="P6" s="8"/>
       <c r="Q6" s="8"/>
       <c r="R6" s="8"/>
-      <c r="S6" s="8"/>
+      <c r="S6" s="1"/>
       <c r="T6" s="1"/>
-      <c r="U6" s="1"/>
+      <c r="AD6" s="3"/>
       <c r="AE6" s="3"/>
       <c r="AF6" s="3"/>
-      <c r="AG6" s="3"/>
-      <c r="AI6" s="3"/>
-    </row>
-    <row r="7" spans="1:38">
-      <c r="I7" s="1"/>
-      <c r="J7" s="2"/>
+    </row>
+    <row r="7" spans="1:36">
+      <c r="H7" s="1"/>
+      <c r="I7" s="2"/>
+      <c r="L7" s="3"/>
       <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="8"/>
+      <c r="S7" s="1"/>
       <c r="T7" s="1"/>
-      <c r="U7" s="1"/>
+      <c r="AD7" s="3"/>
       <c r="AE7" s="3"/>
       <c r="AF7" s="3"/>
-      <c r="AG7" s="3"/>
-      <c r="AI7" s="3"/>
-    </row>
-    <row r="8" spans="1:38">
-      <c r="I8" s="1"/>
-      <c r="J8" s="2"/>
+    </row>
+    <row r="8" spans="1:36">
+      <c r="H8" s="1"/>
+      <c r="I8" s="2"/>
+      <c r="L8" s="3"/>
       <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="8"/>
+      <c r="S8" s="1"/>
       <c r="T8" s="1"/>
-      <c r="U8" s="1"/>
+      <c r="AD8" s="3"/>
       <c r="AE8" s="3"/>
       <c r="AF8" s="3"/>
-      <c r="AG8" s="3"/>
-      <c r="AI8" s="3"/>
-    </row>
-    <row r="9" spans="1:38">
-      <c r="I9" s="1"/>
-      <c r="J9" s="2"/>
+    </row>
+    <row r="9" spans="1:36">
+      <c r="H9" s="1"/>
+      <c r="I9" s="2"/>
+      <c r="L9" s="3"/>
       <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="P9" s="8"/>
       <c r="Q9" s="8"/>
       <c r="R9" s="8"/>
-      <c r="S9" s="8"/>
+      <c r="S9" s="1"/>
       <c r="T9" s="1"/>
-      <c r="U9" s="1"/>
+      <c r="AD9" s="3"/>
       <c r="AE9" s="3"/>
-      <c r="AF9" s="3"/>
-      <c r="AI9" s="3"/>
-    </row>
-    <row r="10" spans="1:38">
-      <c r="I10" s="1"/>
-      <c r="J10" s="2"/>
+    </row>
+    <row r="10" spans="1:36">
+      <c r="H10" s="1"/>
+      <c r="I10" s="2"/>
+      <c r="L10" s="3"/>
       <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="P10" s="8"/>
       <c r="Q10" s="8"/>
       <c r="R10" s="8"/>
-      <c r="S10" s="8"/>
+      <c r="S10" s="1"/>
       <c r="T10" s="1"/>
-      <c r="U10" s="1"/>
+      <c r="AD10" s="3"/>
       <c r="AE10" s="3"/>
-      <c r="AF10" s="3"/>
-      <c r="AI10" s="3"/>
-    </row>
-    <row r="11" spans="1:38">
+    </row>
+    <row r="11" spans="1:36">
+      <c r="P11" s="9"/>
       <c r="Q11" s="9"/>
       <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-    </row>
-    <row r="12" spans="1:38">
+    </row>
+    <row r="12" spans="1:36">
+      <c r="P12" s="9"/>
       <c r="Q12" s="9"/>
       <c r="R12" s="9"/>
-      <c r="S12" s="9"/>
-    </row>
-    <row r="13" spans="1:38">
+    </row>
+    <row r="13" spans="1:36">
+      <c r="P13" s="9"/>
       <c r="Q13" s="9"/>
       <c r="R13" s="9"/>
-      <c r="S13" s="9"/>
-    </row>
-    <row r="14" spans="1:38">
+    </row>
+    <row r="14" spans="1:36">
+      <c r="P14" s="9"/>
       <c r="Q14" s="9"/>
       <c r="R14" s="9"/>
-      <c r="S14" s="9"/>
-    </row>
-    <row r="15" spans="1:38">
+    </row>
+    <row r="15" spans="1:36">
+      <c r="P15" s="9"/>
       <c r="Q15" s="9"/>
       <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-    </row>
-    <row r="16" spans="1:38">
+    </row>
+    <row r="16" spans="1:36">
+      <c r="P16" s="9"/>
       <c r="Q16" s="9"/>
       <c r="R16" s="9"/>
-      <c r="S16" s="9"/>
-    </row>
-    <row r="17" spans="17:19">
+    </row>
+    <row r="17" spans="16:18">
+      <c r="P17" s="9"/>
       <c r="Q17" s="9"/>
       <c r="R17" s="9"/>
-      <c r="S17" s="9"/>
-    </row>
-    <row r="18" spans="17:19">
+    </row>
+    <row r="18" spans="16:18">
+      <c r="P18" s="9"/>
       <c r="Q18" s="9"/>
       <c r="R18" s="9"/>
-      <c r="S18" s="9"/>
-    </row>
-    <row r="19" spans="17:19">
+    </row>
+    <row r="19" spans="16:18">
+      <c r="P19" s="9"/>
       <c r="Q19" s="9"/>
       <c r="R19" s="9"/>
-      <c r="S19" s="9"/>
-    </row>
-    <row r="20" spans="17:19">
+    </row>
+    <row r="20" spans="16:18">
+      <c r="P20" s="9"/>
       <c r="Q20" s="9"/>
       <c r="R20" s="9"/>
-      <c r="S20" s="9"/>
-    </row>
-    <row r="21" spans="17:19">
+    </row>
+    <row r="21" spans="16:18">
+      <c r="P21" s="9"/>
       <c r="Q21" s="9"/>
       <c r="R21" s="9"/>
-      <c r="S21" s="9"/>
-    </row>
-    <row r="22" spans="17:19">
+    </row>
+    <row r="22" spans="16:18">
+      <c r="P22" s="9"/>
       <c r="Q22" s="9"/>
       <c r="R22" s="9"/>
-      <c r="S22" s="9"/>
-    </row>
-    <row r="23" spans="17:19">
+    </row>
+    <row r="23" spans="16:18">
+      <c r="P23" s="9"/>
       <c r="Q23" s="9"/>
       <c r="R23" s="9"/>
-      <c r="S23" s="9"/>
-    </row>
-    <row r="24" spans="17:19">
+    </row>
+    <row r="24" spans="16:18">
+      <c r="P24" s="9"/>
       <c r="Q24" s="9"/>
       <c r="R24" s="9"/>
-      <c r="S24" s="9"/>
-    </row>
-    <row r="25" spans="17:19">
+    </row>
+    <row r="25" spans="16:18">
+      <c r="P25" s="9"/>
       <c r="Q25" s="9"/>
       <c r="R25" s="9"/>
-      <c r="S25" s="9"/>
-    </row>
-    <row r="26" spans="17:19">
+    </row>
+    <row r="26" spans="16:18">
+      <c r="P26" s="9"/>
       <c r="Q26" s="9"/>
       <c r="R26" s="9"/>
-      <c r="S26" s="9"/>
-    </row>
-    <row r="27" spans="17:19">
+    </row>
+    <row r="27" spans="16:18">
+      <c r="P27" s="9"/>
       <c r="Q27" s="9"/>
       <c r="R27" s="9"/>
-      <c r="S27" s="9"/>
-    </row>
-    <row r="28" spans="17:19">
+    </row>
+    <row r="28" spans="16:18">
+      <c r="P28" s="9"/>
       <c r="Q28" s="9"/>
       <c r="R28" s="9"/>
-      <c r="S28" s="9"/>
-    </row>
-    <row r="29" spans="17:19">
+    </row>
+    <row r="29" spans="16:18">
+      <c r="P29" s="9"/>
       <c r="Q29" s="9"/>
       <c r="R29" s="9"/>
-      <c r="S29" s="9"/>
-    </row>
-    <row r="30" spans="17:19">
+    </row>
+    <row r="30" spans="16:18">
+      <c r="P30" s="9"/>
       <c r="Q30" s="9"/>
       <c r="R30" s="9"/>
-      <c r="S30" s="9"/>
-    </row>
-    <row r="31" spans="17:19">
+    </row>
+    <row r="31" spans="16:18">
+      <c r="P31" s="9"/>
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
-      <c r="S31" s="9"/>
-    </row>
-    <row r="32" spans="17:19">
+    </row>
+    <row r="32" spans="16:18">
+      <c r="P32" s="9"/>
       <c r="Q32" s="9"/>
       <c r="R32" s="9"/>
-      <c r="S32" s="9"/>
-    </row>
-    <row r="33" spans="17:19">
+    </row>
+    <row r="33" spans="16:18">
+      <c r="P33" s="9"/>
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
-      <c r="S33" s="9"/>
-    </row>
-    <row r="34" spans="17:19">
+    </row>
+    <row r="34" spans="16:18">
+      <c r="P34" s="9"/>
       <c r="Q34" s="9"/>
       <c r="R34" s="9"/>
-      <c r="S34" s="9"/>
-    </row>
-    <row r="35" spans="17:19">
+    </row>
+    <row r="35" spans="16:18">
+      <c r="P35" s="9"/>
       <c r="Q35" s="9"/>
       <c r="R35" s="9"/>
-      <c r="S35" s="9"/>
-    </row>
-    <row r="36" spans="17:19">
+    </row>
+    <row r="36" spans="16:18">
+      <c r="P36" s="9"/>
       <c r="Q36" s="9"/>
       <c r="R36" s="9"/>
-      <c r="S36" s="9"/>
-    </row>
-    <row r="37" spans="17:19">
+    </row>
+    <row r="37" spans="16:18">
+      <c r="P37" s="9"/>
       <c r="Q37" s="9"/>
       <c r="R37" s="9"/>
-      <c r="S37" s="9"/>
-    </row>
-    <row r="38" spans="17:19">
+    </row>
+    <row r="38" spans="16:18">
+      <c r="P38" s="9"/>
       <c r="Q38" s="9"/>
       <c r="R38" s="9"/>
-      <c r="S38" s="9"/>
-    </row>
-    <row r="39" spans="17:19">
+    </row>
+    <row r="39" spans="16:18">
+      <c r="P39" s="9"/>
       <c r="Q39" s="9"/>
       <c r="R39" s="9"/>
-      <c r="S39" s="9"/>
-    </row>
-    <row r="40" spans="17:19">
+    </row>
+    <row r="40" spans="16:18">
+      <c r="P40" s="9"/>
       <c r="Q40" s="9"/>
       <c r="R40" s="9"/>
-      <c r="S40" s="9"/>
-    </row>
-    <row r="41" spans="17:19">
+    </row>
+    <row r="41" spans="16:18">
+      <c r="P41" s="9"/>
       <c r="Q41" s="9"/>
       <c r="R41" s="9"/>
-      <c r="S41" s="9"/>
-    </row>
-    <row r="42" spans="17:19">
+    </row>
+    <row r="42" spans="16:18">
+      <c r="P42" s="9"/>
       <c r="Q42" s="9"/>
       <c r="R42" s="9"/>
-      <c r="S42" s="9"/>
-    </row>
-    <row r="43" spans="17:19">
+    </row>
+    <row r="43" spans="16:18">
+      <c r="P43" s="9"/>
       <c r="Q43" s="9"/>
       <c r="R43" s="9"/>
-      <c r="S43" s="9"/>
-    </row>
-    <row r="44" spans="17:19">
+    </row>
+    <row r="44" spans="16:18">
+      <c r="P44" s="9"/>
       <c r="Q44" s="9"/>
       <c r="R44" s="9"/>
-      <c r="S44" s="9"/>
-    </row>
-    <row r="45" spans="17:19">
+    </row>
+    <row r="45" spans="16:18">
+      <c r="P45" s="9"/>
       <c r="Q45" s="9"/>
       <c r="R45" s="9"/>
-      <c r="S45" s="9"/>
-    </row>
-    <row r="46" spans="17:19">
+    </row>
+    <row r="46" spans="16:18">
+      <c r="P46" s="9"/>
       <c r="Q46" s="9"/>
       <c r="R46" s="9"/>
-      <c r="S46" s="9"/>
-    </row>
-    <row r="47" spans="17:19">
+    </row>
+    <row r="47" spans="16:18">
+      <c r="P47" s="9"/>
       <c r="Q47" s="9"/>
       <c r="R47" s="9"/>
-      <c r="S47" s="9"/>
-    </row>
-    <row r="48" spans="17:19">
+    </row>
+    <row r="48" spans="16:18">
+      <c r="P48" s="9"/>
       <c r="Q48" s="9"/>
       <c r="R48" s="9"/>
-      <c r="S48" s="9"/>
-    </row>
-    <row r="49" spans="17:19">
+    </row>
+    <row r="49" spans="16:18">
+      <c r="P49" s="9"/>
       <c r="Q49" s="9"/>
       <c r="R49" s="9"/>
-      <c r="S49" s="9"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AK1048576 AL1:AL1048576 AH2:AH1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2:AI1048576 AJ1:AJ1048576 AG2:AG1048576">
       <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="E3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>